<commit_message>
fixed: updated import Question sample question template
</commit_message>
<xml_diff>
--- a/smart_exam_system/static/downloads/sample_question_template.xlsx
+++ b/smart_exam_system/static/downloads/sample_question_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\LMS_PROJECT\AI-Assessment-Platform\smart_exam_system\static\downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A68A557-44ED-4400-8003-56A1C77425E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB07797E-21CF-4873-B811-20E72DA990D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,14 +17,14 @@
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$F$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$J$8</definedName>
   </definedNames>
   <calcPr calcId="145621"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="21">
   <si>
     <t>question</t>
   </si>
@@ -75,6 +75,18 @@
   </si>
   <si>
     <t>3-2=?</t>
+  </si>
+  <si>
+    <t>explanation</t>
+  </si>
+  <si>
+    <t>visual_required</t>
+  </si>
+  <si>
+    <t>visual_type</t>
+  </si>
+  <si>
+    <t>visual</t>
   </si>
 </sst>
 </file>
@@ -154,13 +166,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -183,11 +192,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -493,19 +499,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G76"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="41.90625" style="9" customWidth="1"/>
-    <col min="2" max="2" width="14.7265625" style="6" customWidth="1"/>
-    <col min="3" max="3" width="15.26953125" style="6" customWidth="1"/>
-    <col min="4" max="4" width="14.08984375" style="6" customWidth="1"/>
-    <col min="5" max="5" width="14.453125" style="6" customWidth="1"/>
-    <col min="6" max="6" width="18.81640625" style="11" customWidth="1"/>
-    <col min="7" max="16384" width="8.7265625" style="6"/>
+    <col min="1" max="1" width="41.90625" style="8" customWidth="1"/>
+    <col min="2" max="2" width="14.7265625" style="5" customWidth="1"/>
+    <col min="3" max="3" width="15.26953125" style="5" customWidth="1"/>
+    <col min="4" max="4" width="14.08984375" style="5" customWidth="1"/>
+    <col min="5" max="5" width="14.453125" style="5" customWidth="1"/>
+    <col min="6" max="6" width="18.81640625" style="10" customWidth="1"/>
+    <col min="7" max="7" width="17.26953125" style="5" customWidth="1"/>
+    <col min="8" max="8" width="17.7265625" style="5" customWidth="1"/>
+    <col min="9" max="9" width="16.453125" style="5" customWidth="1"/>
+    <col min="10" max="10" width="12.36328125" style="5" customWidth="1"/>
+    <col min="11" max="16384" width="8.7265625" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -524,386 +534,203 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2"/>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A2" s="12" t="s">
+      <c r="G1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A2" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="B2" s="4">
+      <c r="B2" s="3">
         <v>2</v>
       </c>
-      <c r="C2" s="4">
+      <c r="C2" s="3">
         <v>3</v>
       </c>
-      <c r="D2" s="4">
+      <c r="D2" s="3">
         <v>4</v>
       </c>
-      <c r="E2" s="4">
+      <c r="E2" s="3">
         <v>5</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="5"/>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A3" s="12" t="s">
+      <c r="G2" s="4"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A3" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="4">
+      <c r="B3" s="3">
         <v>2</v>
       </c>
-      <c r="C3" s="4">
+      <c r="C3" s="3">
         <v>7</v>
       </c>
-      <c r="D3" s="4">
+      <c r="D3" s="3">
         <v>4</v>
       </c>
-      <c r="E3" s="4">
+      <c r="E3" s="3">
         <v>5</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G3" s="5"/>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A4" s="12" t="s">
+      <c r="G3" s="4"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A4" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="4">
+      <c r="B4" s="3">
         <v>2</v>
       </c>
-      <c r="C4" s="4">
+      <c r="C4" s="3">
         <v>3</v>
       </c>
-      <c r="D4" s="4">
+      <c r="D4" s="3">
         <v>4</v>
       </c>
-      <c r="E4" s="4">
+      <c r="E4" s="3">
         <v>10</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="G4" s="5"/>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A5" s="12" t="s">
+      <c r="G4" s="4"/>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A5" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="4">
+      <c r="B5" s="3">
         <v>6</v>
       </c>
-      <c r="C5" s="4">
+      <c r="C5" s="3">
         <v>3</v>
       </c>
-      <c r="D5" s="4">
+      <c r="D5" s="3">
         <v>4</v>
       </c>
-      <c r="E5" s="4">
+      <c r="E5" s="3">
         <v>5</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="F5" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="G5" s="5"/>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A6" s="12" t="s">
+      <c r="G5" s="4"/>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A6" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="4">
+      <c r="B6" s="3">
         <v>2</v>
       </c>
-      <c r="C6" s="4">
+      <c r="C6" s="3">
         <v>5</v>
       </c>
-      <c r="D6" s="4">
+      <c r="D6" s="3">
         <v>4</v>
       </c>
-      <c r="E6" s="4">
+      <c r="E6" s="3">
         <v>1</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="F6" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G6" s="5"/>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A7" s="12" t="s">
+      <c r="G6" s="4"/>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A7" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="B7" s="4">
+      <c r="B7" s="3">
         <v>2</v>
       </c>
-      <c r="C7" s="4">
+      <c r="C7" s="3">
         <v>6</v>
       </c>
-      <c r="D7" s="4">
+      <c r="D7" s="3">
         <v>8</v>
       </c>
-      <c r="E7" s="4">
+      <c r="E7" s="3">
         <v>4</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="F7" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="G7" s="5"/>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A8" s="12" t="s">
+      <c r="G7" s="4"/>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A8" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="4">
+      <c r="B8" s="3">
         <v>1</v>
       </c>
-      <c r="C8" s="4">
+      <c r="C8" s="3">
         <v>3</v>
       </c>
-      <c r="D8" s="4">
+      <c r="D8" s="3">
         <v>5</v>
       </c>
-      <c r="E8" s="4">
+      <c r="E8" s="3">
         <v>2</v>
       </c>
-      <c r="F8" s="4" t="s">
+      <c r="F8" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="G8" s="5"/>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A9" s="13"/>
-      <c r="B9" s="7"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="8"/>
-      <c r="G9" s="5"/>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A10" s="13"/>
-      <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="8"/>
-      <c r="G10" s="5"/>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A11" s="13"/>
-      <c r="B11" s="5"/>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
-      <c r="F11" s="8"/>
-      <c r="G11" s="5"/>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A12" s="13"/>
-      <c r="B12" s="5"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
-      <c r="F12" s="8"/>
-      <c r="G12" s="5"/>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A13" s="13"/>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A14" s="13"/>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A15" s="13"/>
-      <c r="C15" s="10"/>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A16" s="13"/>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A17" s="13"/>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A18" s="13"/>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A19" s="13"/>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A20" s="13"/>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A21" s="13"/>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A22" s="13"/>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A23" s="13"/>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A24" s="13"/>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A25" s="13"/>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A26" s="13"/>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A27" s="13"/>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A28" s="13"/>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A29" s="13"/>
-    </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A30" s="13"/>
-    </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A31" s="13"/>
-    </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A32" s="13"/>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A33" s="13"/>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A34" s="13"/>
-    </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A35" s="13"/>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A36" s="13"/>
-    </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A37" s="13"/>
-    </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A38" s="13"/>
-    </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A39" s="13"/>
-    </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A40" s="13"/>
-    </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A41" s="13"/>
-    </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A42" s="13"/>
-    </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A43" s="13"/>
-    </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A44" s="13"/>
-    </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A45" s="13"/>
-    </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A46" s="13"/>
-    </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A47" s="13"/>
-    </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A48" s="13"/>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A49" s="13"/>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A50" s="13"/>
-    </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A51" s="13"/>
-    </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A52" s="13"/>
-    </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A53" s="13"/>
-    </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A54" s="13"/>
-    </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A55" s="13"/>
-    </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A56" s="13"/>
-    </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A57" s="13"/>
-    </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A58" s="13"/>
-    </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A59" s="13"/>
-    </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A60" s="13"/>
-    </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A61" s="13"/>
-    </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A62" s="13"/>
-    </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A63" s="13"/>
-    </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A64" s="13"/>
-    </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A65" s="13"/>
-    </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A66" s="13"/>
-    </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A67" s="13"/>
-    </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A68" s="13"/>
-    </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A69" s="13"/>
-    </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A70" s="13"/>
-    </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A71" s="13"/>
-    </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A72" s="13"/>
-    </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A73" s="13"/>
-    </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A74" s="13"/>
-    </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A75" s="13"/>
-    </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A76" s="13"/>
+      <c r="G8" s="4"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B9" s="6"/>
+      <c r="C9" s="6"/>
+      <c r="D9" s="6"/>
+      <c r="E9" s="6"/>
+      <c r="F9" s="7"/>
+      <c r="G9" s="4"/>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B10" s="4"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4"/>
+      <c r="F10" s="7"/>
+      <c r="G10" s="4"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B11" s="4"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="7"/>
+      <c r="G11" s="4"/>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B12" s="4"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4"/>
+      <c r="F12" s="7"/>
+      <c r="G12" s="4"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="C15" s="9"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F8" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:J8" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>